<commit_message>
Progress bars and examples
</commit_message>
<xml_diff>
--- a/project/PROJECT_X/0_Модели/0.2_Ведомость состава изделия.xlsx
+++ b/project/PROJECT_X/0_Модели/0.2_Ведомость состава изделия.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dmitrii.kriskovets\Desktop\it\5\IDPAM_1.0\project\PROJECT_X\0_Модели\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{393E1F34-5933-43BD-8D52-86B43D4D1021}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1B48E5-046B-4338-A634-4D26DE36F939}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="38400" windowHeight="16755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="56">
   <si>
     <t>Разраб.</t>
   </si>
@@ -194,6 +194,9 @@
   </si>
   <si>
     <t>ООО "МОЯ ОБОРОНА"</t>
+  </si>
+  <si>
+    <t>Деталь</t>
   </si>
 </sst>
 </file>
@@ -1189,7 +1192,7 @@
     <row r="4" spans="1:18" ht="28.5" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="str">
         <f>(IF((E4 = "Пр-во"), (B4 &amp; " - " &amp; C4), C4)) &amp; IF(D4="Сборка", ".iam", ".ipt")</f>
-        <v>PROJECT_X.0002 - Деталь 1.iam</v>
+        <v>PROJECT_X.0002 - Деталь 1.ipt</v>
       </c>
       <c r="B4" s="2" t="str">
         <f>'КВ (установка)'!B7</f>
@@ -1200,7 +1203,7 @@
         <v>Деталь 1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>16</v>

</xml_diff>